<commit_message>
added new class to translate VENDOR_ID to portfolio (approximate)
</commit_message>
<xml_diff>
--- a/PlanStates/VENDOR-PORTFOLIO.xlsx
+++ b/PlanStates/VENDOR-PORTFOLIO.xlsx
@@ -650,10 +650,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="K3" t="s">
         <v>29</v>
@@ -664,10 +664,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="K4" t="s">
         <v>30</v>
@@ -678,10 +678,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="K5" t="s">
         <v>31</v>
@@ -692,10 +692,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="K6" t="s">
         <v>32</v>
@@ -706,21 +706,24 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>2</v>
       </c>
       <c r="K7" t="s">
         <v>33</v>
       </c>
+      <c r="L7">
+        <v>9999</v>
+      </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K8" t="s">
         <v>34</v>
@@ -731,10 +734,10 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K9" t="s">
         <v>35</v>
@@ -745,10 +748,10 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="K10" t="s">
         <v>36</v>
@@ -759,21 +762,24 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="K11" t="s">
         <v>37</v>
       </c>
+      <c r="L11">
+        <v>11</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="K12" t="s">
         <v>38</v>
@@ -784,21 +790,24 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="K13" t="s">
         <v>39</v>
       </c>
+      <c r="L13">
+        <v>9999</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="K14" t="s">
         <v>40</v>
@@ -809,10 +818,10 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="K15" t="s">
         <v>41</v>
@@ -823,10 +832,10 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="K16" t="s">
         <v>42</v>
@@ -837,10 +846,10 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="K17" t="s">
         <v>43</v>
@@ -851,43 +860,52 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="K18" t="s">
         <v>44</v>
       </c>
+      <c r="L18">
+        <v>15</v>
+      </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K19" t="s">
         <v>45</v>
       </c>
+      <c r="L19">
+        <v>12</v>
+      </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="K20" t="s">
         <v>46</v>
       </c>
+      <c r="L20">
+        <v>25</v>
+      </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="K21" t="s">
         <v>47</v>
@@ -898,10 +916,10 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="K22" t="s">
         <v>48</v>
@@ -912,10 +930,10 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K23" t="s">
         <v>49</v>
@@ -926,10 +944,10 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="K24" t="s">
         <v>50</v>
@@ -940,81 +958,117 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="K25" t="s">
         <v>51</v>
       </c>
+      <c r="L25">
+        <v>9999</v>
+      </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="K26" t="s">
         <v>52</v>
       </c>
+      <c r="L26">
+        <v>9999</v>
+      </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K27" t="s">
         <v>53</v>
+      </c>
+      <c r="L27">
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K28" t="s">
         <v>54</v>
       </c>
+      <c r="L28">
+        <v>2</v>
+      </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K29" t="s">
         <v>55</v>
       </c>
+      <c r="L29">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K30" t="s">
         <v>56</v>
       </c>
+      <c r="L30">
+        <v>2</v>
+      </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K31" t="s">
         <v>57</v>
       </c>
+      <c r="L31">
+        <v>24</v>
+      </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="K32" t="s">
         <v>58</v>
       </c>
+      <c r="L32">
+        <v>18</v>
+      </c>
     </row>
     <row r="33" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K33" t="s">
         <v>59</v>
       </c>
+      <c r="L33">
+        <v>18</v>
+      </c>
     </row>
     <row r="34" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K34" t="s">
         <v>60</v>
       </c>
+      <c r="L34">
+        <v>25</v>
+      </c>
     </row>
     <row r="35" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K35" t="s">
         <v>61</v>
       </c>
+      <c r="L35">
+        <v>24</v>
+      </c>
     </row>
     <row r="36" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K36" t="s">
         <v>62</v>
       </c>
+      <c r="L36">
+        <v>9999</v>
+      </c>
     </row>
     <row r="37" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K37" t="s">
@@ -1068,16 +1122,25 @@
       <c r="K43" t="s">
         <v>69</v>
       </c>
+      <c r="L43">
+        <v>9999</v>
+      </c>
     </row>
     <row r="44" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K44" t="s">
         <v>70</v>
       </c>
+      <c r="L44">
+        <v>9999</v>
+      </c>
     </row>
     <row r="45" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K45" t="s">
         <v>71</v>
       </c>
+      <c r="L45">
+        <v>9999</v>
+      </c>
     </row>
     <row r="46" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K46" t="s">
@@ -1107,11 +1170,17 @@
       <c r="K49" t="s">
         <v>10</v>
       </c>
+      <c r="L49">
+        <v>5</v>
+      </c>
     </row>
     <row r="50" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K50" t="s">
         <v>75</v>
       </c>
+      <c r="L50">
+        <v>5</v>
+      </c>
     </row>
     <row r="51" spans="11:12" x14ac:dyDescent="0.25">
       <c r="K51" t="s">
@@ -1139,7 +1208,7 @@
     </row>
   </sheetData>
   <sortState ref="A2:B27">
-    <sortCondition ref="B2:B27"/>
+    <sortCondition ref="A2:A27"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>